<commit_message>
Formel an Excel-Blatt berechnung_fertig angepasst
Saettigungsdruck 0.52 + 0.07*T (vorher 0.51 + 0.076*T) und
Kuehlschlange als Wert 14 ohne zusaetzliches *0.05.
SW-Cache auf v3 erhoeht, damit installierte PWAs aktualisieren.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Druckberechnung_CO2_4_Biere.xlsx
+++ b/Druckberechnung_CO2_4_Biere.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30219"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://schlosseggenbergat.sharepoint.com/sites/TechnischerKundendienst/Freigegebene Dokumente/Allgemein/Schanktechnik/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="58" documentId="8_{E47063D8-7BD0-4758-8BC3-39F1BFEFC615}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E7124752-14A4-44A8-B834-75C026F4267B}"/>
+  <xr:revisionPtr revIDLastSave="128" documentId="8_{E47063D8-7BD0-4758-8BC3-39F1BFEFC615}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4D2CCA3F-5CD4-4B6E-8BCC-4D55E40D3BB8}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="4425" yWindow="1530" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="4425" yWindow="1530" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Druckberechnung_4_Biere" sheetId="1" r:id="rId1"/>
+    <sheet name="berechnung_fertig" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="19">
   <si>
     <t>Bier</t>
   </si>
@@ -86,20 +87,20 @@
     <t>Bier 2</t>
   </si>
   <si>
+    <t>ja</t>
+  </si>
+  <si>
     <t>Bier 3</t>
   </si>
   <si>
     <t>Bier 4</t>
-  </si>
-  <si>
-    <t>ja</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -451,14 +452,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D32"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="29" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="7.5703125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="21" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" ht="21">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -472,7 +473,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -480,25 +481,25 @@
         <v>5</v>
       </c>
       <c r="C2" s="1">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4">
       <c r="B3" t="s">
         <v>7</v>
       </c>
       <c r="C3">
         <f>0.51 + 0.076*C2</f>
-        <v>1.27</v>
+        <v>0.96599999999999997</v>
       </c>
       <c r="D3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4">
       <c r="B4" t="s">
         <v>9</v>
       </c>
@@ -509,26 +510,24 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4">
       <c r="B5" t="s">
         <v>11</v>
       </c>
       <c r="C5" s="1">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="D5" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4">
       <c r="B6" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C6" s="1"/>
+    </row>
+    <row r="7" spans="1:4">
       <c r="B7" t="s">
         <v>13</v>
       </c>
@@ -539,93 +538,100 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4">
       <c r="B8" t="s">
         <v>14</v>
       </c>
       <c r="C8">
         <f>C3 + 0.1*C4 + 0.05*(C5 + C7*0.05)</f>
-        <v>1.87</v>
+        <v>1.1160000000000001</v>
       </c>
       <c r="D8" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4">
       <c r="A10" t="s">
         <v>15</v>
       </c>
       <c r="B10" t="s">
         <v>5</v>
       </c>
-      <c r="C10" s="1"/>
+      <c r="C10" s="1">
+        <v>30</v>
+      </c>
       <c r="D10" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4">
       <c r="B11" t="s">
         <v>7</v>
       </c>
       <c r="C11">
         <f>0.52 + 0.065*C10</f>
-        <v>0.52</v>
+        <v>2.4700000000000002</v>
       </c>
       <c r="D11" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4">
       <c r="B12" t="s">
         <v>9</v>
       </c>
-      <c r="C12" s="1"/>
+      <c r="C12" s="1">
+        <v>1</v>
+      </c>
       <c r="D12" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4">
       <c r="B13" t="s">
         <v>11</v>
       </c>
-      <c r="C13" s="1"/>
+      <c r="C13" s="1">
+        <v>1</v>
+      </c>
       <c r="D13" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4">
       <c r="B14" t="s">
         <v>12</v>
       </c>
-      <c r="C14" s="1"/>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C14" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4">
       <c r="B15" t="s">
         <v>13</v>
       </c>
       <c r="C15">
-        <f>IF(C14="ja",14,0)</f>
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="D15" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4">
       <c r="B16" t="s">
         <v>14</v>
       </c>
       <c r="C16">
         <f>C11 + 0.1*C12 + 0.05*(C13 + C15)</f>
-        <v>0.52</v>
+        <v>3.3200000000000003</v>
       </c>
       <c r="D16" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4">
       <c r="A18" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B18" t="s">
         <v>5</v>
@@ -635,7 +641,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4">
       <c r="B19" t="s">
         <v>7</v>
       </c>
@@ -647,7 +653,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4">
       <c r="B20" t="s">
         <v>9</v>
       </c>
@@ -656,7 +662,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4">
       <c r="B21" t="s">
         <v>11</v>
       </c>
@@ -665,13 +671,13 @@
         <v>10</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4">
       <c r="B22" t="s">
         <v>12</v>
       </c>
       <c r="C22" s="1"/>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4">
       <c r="B23" t="s">
         <v>13</v>
       </c>
@@ -683,7 +689,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4">
       <c r="B24" t="s">
         <v>14</v>
       </c>
@@ -695,9 +701,9 @@
         <v>8</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4">
       <c r="A26" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B26" t="s">
         <v>5</v>
@@ -707,7 +713,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4">
       <c r="B27" t="s">
         <v>7</v>
       </c>
@@ -719,7 +725,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4">
       <c r="B28" t="s">
         <v>9</v>
       </c>
@@ -728,7 +734,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4">
       <c r="B29" t="s">
         <v>11</v>
       </c>
@@ -737,13 +743,13 @@
         <v>10</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4">
       <c r="B30" t="s">
         <v>12</v>
       </c>
       <c r="C30" s="1"/>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4">
       <c r="B31" t="s">
         <v>13</v>
       </c>
@@ -755,7 +761,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4">
       <c r="B32" t="s">
         <v>14</v>
       </c>
@@ -772,16 +778,100 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB8DAAD5-A999-47DB-A0DE-672F0AB7562B}">
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="2" max="2" width="28.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="1">
+        <v>6</v>
+      </c>
+      <c r="D1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="B2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2">
+        <f>0.52 + 0.07*C1</f>
+        <v>0.94000000000000006</v>
+      </c>
+      <c r="D2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="B3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="1">
+        <v>1</v>
+      </c>
+      <c r="D3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="B4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="1">
+        <v>1</v>
+      </c>
+      <c r="D4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="B5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="B6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6">
+        <f>IF(C5="ja",14,0)</f>
+        <v>14</v>
+      </c>
+      <c r="D6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="B7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7">
+        <f>C2 + 0.1*C3 + 0.05*(C4 + C6)</f>
+        <v>1.79</v>
+      </c>
+      <c r="D7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100EBE6B5A6B738C446A94CBD495F919F11" ma:contentTypeVersion="11" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="b679d2dd8dfd8e08f4c04c3dae124ed1">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="21682ff3-ec6b-4905-98b2-53709a7e75ac" xmlns:ns3="f5a45939-d3bc-454c-acab-6d02ab4fc35f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="bb8fc6d53e3ad405423d7545b4ed343f" ns2:_="" ns3:_="">
     <xsd:import namespace="21682ff3-ec6b-4905-98b2-53709a7e75ac"/>
@@ -976,6 +1066,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -988,39 +1087,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F972A06B-AAED-40EC-9115-9097C280291F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F3C8283-AC58-49C0-820C-245828275CCD}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F3C8283-AC58-49C0-820C-245828275CCD}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="21682ff3-ec6b-4905-98b2-53709a7e75ac"/>
-    <ds:schemaRef ds:uri="f5a45939-d3bc-454c-acab-6d02ab4fc35f"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F972A06B-AAED-40EC-9115-9097C280291F}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4983E224-D53A-4EB3-9EF9-9B2FACCF6D27}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="f5a45939-d3bc-454c-acab-6d02ab4fc35f"/>
-    <ds:schemaRef ds:uri="21682ff3-ec6b-4905-98b2-53709a7e75ac"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4983E224-D53A-4EB3-9EF9-9B2FACCF6D27}"/>
 </file>
</xml_diff>